<commit_message>
Gridfinity box config clean ups.
</commit_message>
<xml_diff>
--- a/Equasions.xlsx
+++ b/Equasions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Waterproof_Box_CAD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_Local\Waterproof_Box_CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487E9C28-CAD6-4780-B6CC-E76BC4AB5F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27BA3480-B36A-45E2-A38F-09AD0813757E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" firstSheet="18" activeTab="19" xr2:uid="{183B79F6-9E5A-40E4-98DA-2846F6A131E3}"/>
+    <workbookView xWindow="40290" yWindow="2540" windowWidth="29450" windowHeight="16220" firstSheet="20" activeTab="27" xr2:uid="{183B79F6-9E5A-40E4-98DA-2846F6A131E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Cash Box" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="104">
   <si>
     <t>Clearance Hole Diameter</t>
   </si>
@@ -361,6 +361,9 @@
   </si>
   <si>
     <t>66.7mm</t>
+  </si>
+  <si>
+    <t>total depth</t>
   </si>
 </sst>
 </file>
@@ -713,19 +716,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21F7FC21-9959-49FE-A5FE-8F450290E594}">
   <dimension ref="A2:D24"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -739,7 +742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -753,7 +756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -767,7 +770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -781,7 +784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -795,7 +798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -809,7 +812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -823,7 +826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -837,7 +840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -851,7 +854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -865,7 +868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -879,7 +882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -893,7 +896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -907,27 +910,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -942,7 +945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -957,17 +960,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -980,20 +983,20 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53E3CC92-C677-4B52-9418-CD6D075FABE4}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1007,7 +1010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1021,7 +1024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1035,7 +1038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1049,7 +1052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1063,7 +1066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1077,7 +1080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1091,7 +1094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1105,7 +1108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1119,7 +1122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1133,7 +1136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1147,7 +1150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1161,7 +1164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1175,27 +1178,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1210,7 +1213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1225,7 +1228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1249,20 +1252,20 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6231AABF-8B48-447F-85FB-DE1948E7B094}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1276,7 +1279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1290,7 +1293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1304,7 +1307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1318,7 +1321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1332,7 +1335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1346,7 +1349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1360,7 +1363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1374,7 +1377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1388,7 +1391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1402,7 +1405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1416,7 +1419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1430,7 +1433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1444,27 +1447,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1479,7 +1482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1494,7 +1497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1502,7 +1505,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1518,20 +1521,20 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16A8E5B-6D41-447C-B97A-46BCD234EBD3}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1545,7 +1548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1559,7 +1562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1573,7 +1576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1587,7 +1590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1601,7 +1604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1615,7 +1618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1629,7 +1632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1643,7 +1646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1657,7 +1660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1671,7 +1674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1685,7 +1688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1699,7 +1702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1713,27 +1716,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1748,7 +1751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1763,7 +1766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1771,7 +1774,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1787,20 +1790,20 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B99A14FA-F64C-436A-BEBE-7B3B6267FFE1}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1814,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1828,7 +1831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1842,7 +1845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1856,7 +1859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1870,7 +1873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1884,7 +1887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1898,7 +1901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1912,7 +1915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1926,7 +1929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1940,7 +1943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1954,7 +1957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1968,7 +1971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1982,27 +1985,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -2017,7 +2020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -2032,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -2040,7 +2043,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -2056,15 +2059,15 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{310D36E6-7104-47E8-997B-24650DC8E3D9}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2078,7 +2081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2092,7 +2095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2106,7 +2109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2120,7 +2123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -2134,7 +2137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2148,7 +2151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2162,7 +2165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2176,7 +2179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -2190,7 +2193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -2204,7 +2207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2218,7 +2221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2232,7 +2235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2246,27 +2249,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -2281,7 +2284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -2296,7 +2299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -2304,7 +2307,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -2320,15 +2323,15 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FEE99C3-AEF2-482F-B05F-EFD41E7E2C81}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2342,7 +2345,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2356,7 +2359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2370,7 +2373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2384,7 +2387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -2398,7 +2401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2412,7 +2415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2426,7 +2429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2440,7 +2443,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -2454,7 +2457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -2468,7 +2471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2482,7 +2485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2496,7 +2499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2510,27 +2513,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -2545,7 +2548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -2560,7 +2563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -2568,7 +2571,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -2584,20 +2587,20 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD0F985-F179-4AB5-94A8-A2BDB2643FEF}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2611,7 +2614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2625,7 +2628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2639,7 +2642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2653,7 +2656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2667,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2681,7 +2684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2695,7 +2698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2709,7 +2712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2723,7 +2726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -2737,7 +2740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -2751,7 +2754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -2765,7 +2768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -2779,7 +2782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -2787,7 +2790,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2803,20 +2806,20 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5BBFB27-C2D1-4A50-B307-C272938C9950}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2830,7 +2833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2844,7 +2847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2858,7 +2861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2872,7 +2875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2886,7 +2889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2900,7 +2903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2914,7 +2917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2928,7 +2931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2942,7 +2945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -2956,7 +2959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -2970,7 +2973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -2984,7 +2987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -2998,7 +3001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -3006,7 +3009,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>83</v>
       </c>
@@ -3022,20 +3025,20 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F100B82-B81A-48EF-BF19-D32B8C772AD2}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3049,7 +3052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3063,7 +3066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3077,7 +3080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3091,7 +3094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3105,7 +3108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3119,7 +3122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3133,7 +3136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3147,7 +3150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3161,7 +3164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3175,7 +3178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3189,7 +3192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3203,7 +3206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3225,20 +3228,20 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3599EF72-21DF-47D8-B50B-70E6A87BD8DA}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3252,7 +3255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3266,7 +3269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3280,7 +3283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3294,7 +3297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3308,7 +3311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3322,7 +3325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3336,7 +3339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3350,7 +3353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3364,7 +3367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3378,7 +3381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3392,7 +3395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3406,7 +3409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3420,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -3436,20 +3439,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FAAAC63-42B8-45C9-A7F0-088070DACEA1}">
   <dimension ref="A1:D28"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3463,7 +3466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3477,7 +3480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3491,7 +3494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3505,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3519,7 +3522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3533,7 +3536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3547,7 +3550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3561,7 +3564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3575,7 +3578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3589,7 +3592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3603,7 +3606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3617,7 +3620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3631,27 +3634,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -3666,7 +3669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -3681,22 +3684,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -3704,7 +3707,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3712,7 +3715,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>73</v>
       </c>
@@ -3720,7 +3723,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>75</v>
       </c>
@@ -3736,20 +3739,20 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99E881B5-3D64-499C-A9D0-333A76B0ED05}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3763,7 +3766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3777,7 +3780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3791,7 +3794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3805,7 +3808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3819,7 +3822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3833,7 +3836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3847,7 +3850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3861,7 +3864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3875,7 +3878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3889,7 +3892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3903,7 +3906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3917,7 +3920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3931,7 +3934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -3939,7 +3942,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -3955,20 +3958,20 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B6511CC-38E1-4154-B821-2D6A4449464B}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3982,7 +3985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3996,7 +3999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4010,7 +4013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4024,7 +4027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4038,7 +4041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4052,7 +4055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4066,7 +4069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4080,7 +4083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4094,7 +4097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4108,7 +4111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4122,7 +4125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4136,7 +4139,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4150,7 +4153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4166,20 +4169,20 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49CF470F-97CD-4075-8C0A-E3E45C00CC04}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4193,7 +4196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4207,7 +4210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4221,7 +4224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4235,7 +4238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4249,7 +4252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4263,7 +4266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4277,7 +4280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4291,7 +4294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4305,7 +4308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4319,7 +4322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4333,7 +4336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4347,7 +4350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4361,7 +4364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4377,20 +4380,20 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54ED4996-851A-4029-8EF7-FDBF014DE0C1}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4404,7 +4407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4418,7 +4421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4432,7 +4435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4446,7 +4449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4460,7 +4463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4474,7 +4477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4488,7 +4491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4502,7 +4505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4516,7 +4519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4530,7 +4533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4544,7 +4547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4558,7 +4561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4572,7 +4575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4588,20 +4591,20 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AC6754A-E88D-459A-BAB5-89402A897BF9}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4615,7 +4618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4629,7 +4632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4643,7 +4646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4657,7 +4660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4671,7 +4674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4685,7 +4688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4699,7 +4702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4713,7 +4716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4727,7 +4730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4741,7 +4744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4755,7 +4758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4769,7 +4772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4791,20 +4794,20 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFC1693C-4903-454A-808D-6E40890C47F7}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4818,7 +4821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4832,7 +4835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4846,7 +4849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4860,7 +4863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4874,7 +4877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4888,7 +4891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4902,7 +4905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4916,7 +4919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4930,7 +4933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4944,7 +4947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4958,7 +4961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4972,7 +4975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4986,7 +4989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4994,7 +4997,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -5010,17 +5013,17 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00F2F41-2390-4D5B-87F0-6BC9922397BA}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5034,7 +5037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5048,7 +5051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5062,7 +5065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5076,7 +5079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5090,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5104,7 +5107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5118,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5132,7 +5135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5146,7 +5149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5160,7 +5163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5174,7 +5177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5188,7 +5191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5202,7 +5205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -5218,20 +5221,20 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F70EC75-25B8-4079-A586-BB24271F7259}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5245,7 +5248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5259,7 +5262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5273,7 +5276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5287,7 +5290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5301,7 +5304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5315,7 +5318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5329,7 +5332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5343,7 +5346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5357,7 +5360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5371,7 +5374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5385,7 +5388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5399,7 +5402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5413,7 +5416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -5428,18 +5431,18 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B232E5-FCDB-4A5B-8438-DC7E4074B16B}">
-  <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5453,7 +5456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5467,7 +5470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5481,7 +5484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5495,7 +5498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5509,7 +5512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5523,7 +5526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5537,7 +5540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5551,7 +5554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5565,7 +5568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5579,7 +5582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5593,7 +5596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5607,7 +5610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5621,12 +5624,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>101</v>
       </c>
       <c r="B16" t="s">
         <v>102</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17">
+        <v>74.7</v>
       </c>
     </row>
   </sheetData>
@@ -5637,20 +5648,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B063A3DA-1C44-4C3A-8C1B-E2761804D2D3}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5664,7 +5675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5678,7 +5689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5692,7 +5703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5706,7 +5717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5720,7 +5731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5734,7 +5745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5748,7 +5759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5762,7 +5773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5776,7 +5787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5790,7 +5801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5804,7 +5815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5818,7 +5829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5832,27 +5843,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -5867,7 +5878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -5882,7 +5893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -5890,7 +5901,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -5906,20 +5917,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E85C9EF-C938-4332-9062-B90E5391A4C9}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5933,7 +5944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5947,7 +5958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5961,7 +5972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5975,7 +5986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5989,7 +6000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6003,7 +6014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6017,7 +6028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6031,7 +6042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -6045,7 +6056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -6059,7 +6070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -6073,7 +6084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6087,7 +6098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -6101,27 +6112,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -6136,7 +6147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -6151,7 +6162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -6159,7 +6170,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -6175,20 +6186,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360362D6-FEDB-4209-B94A-90E1261C03E2}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6202,7 +6213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -6216,7 +6227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -6230,7 +6241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -6244,7 +6255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -6258,7 +6269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6272,7 +6283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6286,7 +6297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6300,7 +6311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -6314,7 +6325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -6328,7 +6339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -6342,7 +6353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6356,7 +6367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -6370,27 +6381,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -6405,7 +6416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -6420,7 +6431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -6428,7 +6439,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -6444,20 +6455,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B113761-7CD5-4A92-9B63-87C14A162C82}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6471,7 +6482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -6485,7 +6496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -6499,7 +6510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -6513,7 +6524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -6527,7 +6538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6541,7 +6552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6555,7 +6566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6569,7 +6580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -6583,7 +6594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -6597,7 +6608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -6611,7 +6622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6625,7 +6636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -6639,27 +6650,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -6674,7 +6685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -6689,7 +6700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -6697,7 +6708,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -6713,15 +6724,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B4DCC9-BAEB-4BE3-8071-9749F432ADAE}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6735,7 +6746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -6749,7 +6760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6763,7 +6774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -6777,7 +6788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -6791,7 +6802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -6805,7 +6816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -6819,7 +6830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -6833,7 +6844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -6847,7 +6858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -6861,7 +6872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -6875,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -6889,7 +6900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -6903,27 +6914,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -6938,7 +6949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -6953,7 +6964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -6961,7 +6972,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -6977,20 +6988,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B7BCB8-2BE9-44FE-9BA0-E5BC0BEA7660}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -7004,7 +7015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -7018,7 +7029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -7032,7 +7043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -7046,7 +7057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7060,7 +7071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -7074,7 +7085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -7088,7 +7099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -7102,7 +7113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -7116,7 +7127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -7130,7 +7141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -7144,7 +7155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -7158,7 +7169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -7172,27 +7183,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -7207,7 +7218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -7222,7 +7233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -7230,7 +7241,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -7246,20 +7257,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C644951-C62A-48BD-BE1E-F3508FF13797}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -7273,7 +7284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -7287,7 +7298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -7301,7 +7312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -7315,7 +7326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7329,7 +7340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -7343,7 +7354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -7357,7 +7368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -7371,7 +7382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -7385,7 +7396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -7399,7 +7410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -7413,7 +7424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -7427,7 +7438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -7441,27 +7452,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -7476,7 +7487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -7491,7 +7502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -7499,7 +7510,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>

</xml_diff>

<commit_message>
Uno show em no mercy finished.
</commit_message>
<xml_diff>
--- a/Equasions.xlsx
+++ b/Equasions.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_Local\Waterproof_Box_CAD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT_local\Waterproof_Box_CAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27BA3480-B36A-45E2-A38F-09AD0813757E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{487E9C28-CAD6-4780-B6CC-E76BC4AB5F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40290" yWindow="2540" windowWidth="29450" windowHeight="16220" firstSheet="20" activeTab="27" xr2:uid="{183B79F6-9E5A-40E4-98DA-2846F6A131E3}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18120" firstSheet="18" activeTab="19" xr2:uid="{183B79F6-9E5A-40E4-98DA-2846F6A131E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Cash Box" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="103">
   <si>
     <t>Clearance Hole Diameter</t>
   </si>
@@ -361,9 +361,6 @@
   </si>
   <si>
     <t>66.7mm</t>
-  </si>
-  <si>
-    <t>total depth</t>
   </si>
 </sst>
 </file>
@@ -716,19 +713,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21F7FC21-9959-49FE-A5FE-8F450290E594}">
   <dimension ref="A2:D24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -742,7 +739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -756,7 +753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -770,7 +767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -784,7 +781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -798,7 +795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -812,7 +809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -826,7 +823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -840,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -854,7 +851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -868,7 +865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -882,7 +879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -896,7 +893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -910,27 +907,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -945,7 +942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>39</v>
       </c>
@@ -960,17 +957,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -983,20 +980,20 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53E3CC92-C677-4B52-9418-CD6D075FABE4}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1010,7 +1007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1024,7 +1021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1038,7 +1035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1052,7 +1049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1066,7 +1063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1080,7 +1077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1094,7 +1091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1108,7 +1105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1122,7 +1119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1136,7 +1133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1150,7 +1147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1164,7 +1161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1178,27 +1175,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1213,7 +1210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1228,7 +1225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1236,7 +1233,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1252,20 +1249,20 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6231AABF-8B48-447F-85FB-DE1948E7B094}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1279,7 +1276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1293,7 +1290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1307,7 +1304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1321,7 +1318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1335,7 +1332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1349,7 +1346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1363,7 +1360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1377,7 +1374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1391,7 +1388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1405,7 +1402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1419,7 +1416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1433,7 +1430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1447,27 +1444,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1482,7 +1479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1497,7 +1494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1505,7 +1502,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1521,20 +1518,20 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16A8E5B-6D41-447C-B97A-46BCD234EBD3}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1548,7 +1545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1562,7 +1559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1576,7 +1573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1590,7 +1587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1604,7 +1601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1618,7 +1615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1632,7 +1629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1646,7 +1643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1660,7 +1657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1674,7 +1671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1688,7 +1685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1702,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1716,27 +1713,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1751,7 +1748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1766,7 +1763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -1774,7 +1771,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1790,20 +1787,20 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B99A14FA-F64C-436A-BEBE-7B3B6267FFE1}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1817,7 +1814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -1831,7 +1828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -1845,7 +1842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1859,7 +1856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -1873,7 +1870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1887,7 +1884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1901,7 +1898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1915,7 +1912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1929,7 +1926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1943,7 +1940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -1957,7 +1954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1971,7 +1968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1985,27 +1982,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -2020,7 +2017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -2035,7 +2032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -2043,7 +2040,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -2059,15 +2056,15 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{310D36E6-7104-47E8-997B-24650DC8E3D9}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2081,7 +2078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2095,7 +2092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2109,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2123,7 +2120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -2137,7 +2134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2151,7 +2148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2165,7 +2162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2179,7 +2176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -2193,7 +2190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -2207,7 +2204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2221,7 +2218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2235,7 +2232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2249,27 +2246,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -2284,7 +2281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -2299,7 +2296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -2307,7 +2304,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -2323,15 +2320,15 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FEE99C3-AEF2-482F-B05F-EFD41E7E2C81}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2345,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2359,7 +2356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2373,7 +2370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -2387,7 +2384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -2401,7 +2398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -2415,7 +2412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -2429,7 +2426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -2443,7 +2440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -2457,7 +2454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -2471,7 +2468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -2485,7 +2482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -2499,7 +2496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2513,27 +2510,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -2548,7 +2545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -2563,7 +2560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -2571,7 +2568,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -2587,20 +2584,20 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD0F985-F179-4AB5-94A8-A2BDB2643FEF}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2614,7 +2611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2628,7 +2625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2642,7 +2639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2656,7 +2653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2670,7 +2667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2684,7 +2681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2698,7 +2695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2712,7 +2709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2726,7 +2723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -2740,7 +2737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -2754,7 +2751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -2768,7 +2765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -2782,7 +2779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -2790,7 +2787,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2806,20 +2803,20 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5BBFB27-C2D1-4A50-B307-C272938C9950}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2833,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2847,7 +2844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2861,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2875,7 +2872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -2889,7 +2886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2903,7 +2900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -2917,7 +2914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2931,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2945,7 +2942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -2959,7 +2956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -2973,7 +2970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -2987,7 +2984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3001,7 +2998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -3009,7 +3006,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>83</v>
       </c>
@@ -3025,20 +3022,20 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F100B82-B81A-48EF-BF19-D32B8C772AD2}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3052,7 +3049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3066,7 +3063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3080,7 +3077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3094,7 +3091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3108,7 +3105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3122,7 +3119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3136,7 +3133,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3150,7 +3147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3164,7 +3161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3178,7 +3175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3192,7 +3189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3206,7 +3203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3228,20 +3225,20 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3599EF72-21DF-47D8-B50B-70E6A87BD8DA}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3255,7 +3252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3269,7 +3266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3283,7 +3280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3297,7 +3294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3311,7 +3308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3325,7 +3322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3339,7 +3336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3353,7 +3350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3367,7 +3364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3381,7 +3378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3395,7 +3392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3409,7 +3406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3423,7 +3420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -3439,20 +3436,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FAAAC63-42B8-45C9-A7F0-088070DACEA1}">
   <dimension ref="A1:D28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3466,7 +3463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3480,7 +3477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3494,7 +3491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3508,7 +3505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3522,7 +3519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3536,7 +3533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3550,7 +3547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3564,7 +3561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3578,7 +3575,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3592,7 +3589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3606,7 +3603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3620,7 +3617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3634,27 +3631,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -3669,7 +3666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -3684,22 +3681,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -3707,7 +3704,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3715,7 +3712,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>73</v>
       </c>
@@ -3723,7 +3720,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>75</v>
       </c>
@@ -3739,20 +3736,20 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99E881B5-3D64-499C-A9D0-333A76B0ED05}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3766,7 +3763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3780,7 +3777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -3794,7 +3791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3808,7 +3805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -3822,7 +3819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -3836,7 +3833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3850,7 +3847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3864,7 +3861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -3878,7 +3875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3892,7 +3889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3906,7 +3903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -3920,7 +3917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -3934,7 +3931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -3942,7 +3939,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -3958,20 +3955,20 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B6511CC-38E1-4154-B821-2D6A4449464B}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -3985,7 +3982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -3999,7 +3996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4013,7 +4010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4027,7 +4024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4041,7 +4038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4055,7 +4052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4069,7 +4066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4083,7 +4080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4097,7 +4094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4111,7 +4108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4125,7 +4122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4139,7 +4136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4153,7 +4150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4169,20 +4166,20 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49CF470F-97CD-4075-8C0A-E3E45C00CC04}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4196,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4210,7 +4207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4224,7 +4221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4238,7 +4235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4252,7 +4249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4266,7 +4263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4280,7 +4277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4294,7 +4291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4308,7 +4305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4322,7 +4319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4336,7 +4333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4350,7 +4347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4364,7 +4361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4380,20 +4377,20 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54ED4996-851A-4029-8EF7-FDBF014DE0C1}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4407,7 +4404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4421,7 +4418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4435,7 +4432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4449,7 +4446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4463,7 +4460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4477,7 +4474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4491,7 +4488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4505,7 +4502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4519,7 +4516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4533,7 +4530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4547,7 +4544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4561,7 +4558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4575,7 +4572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4591,20 +4588,20 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AC6754A-E88D-459A-BAB5-89402A897BF9}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4618,7 +4615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4632,7 +4629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4646,7 +4643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4660,7 +4657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4674,7 +4671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4688,7 +4685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4702,7 +4699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4716,7 +4713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4730,7 +4727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4744,7 +4741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4758,7 +4755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4772,7 +4769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4794,20 +4791,20 @@
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFC1693C-4903-454A-808D-6E40890C47F7}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -4821,7 +4818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -4835,7 +4832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -4849,7 +4846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -4863,7 +4860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -4877,7 +4874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -4891,7 +4888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -4905,7 +4902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -4919,7 +4916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -4933,7 +4930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -4947,7 +4944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -4961,7 +4958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -4975,7 +4972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -4989,7 +4986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -4997,7 +4994,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -5013,17 +5010,17 @@
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00F2F41-2390-4D5B-87F0-6BC9922397BA}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5037,7 +5034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5051,7 +5048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5065,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5079,7 +5076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5093,7 +5090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5107,7 +5104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5121,7 +5118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5135,7 +5132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5149,7 +5146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5163,7 +5160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5177,7 +5174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5191,7 +5188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5205,7 +5202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -5221,20 +5218,20 @@
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F70EC75-25B8-4079-A586-BB24271F7259}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5248,7 +5245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5262,7 +5259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5276,7 +5273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5290,7 +5287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5304,7 +5301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5318,7 +5315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5332,7 +5329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5346,7 +5343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5360,7 +5357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5374,7 +5371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5388,7 +5385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5402,7 +5399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5416,7 +5413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>71</v>
       </c>
@@ -5431,18 +5428,18 @@
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63B232E5-FCDB-4A5B-8438-DC7E4074B16B}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5456,7 +5453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5470,7 +5467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5484,7 +5481,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5498,7 +5495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5512,7 +5509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5526,7 +5523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5540,7 +5537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5554,7 +5551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5568,7 +5565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5582,7 +5579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5596,7 +5593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5610,7 +5607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5624,20 +5621,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>101</v>
       </c>
       <c r="B16" t="s">
         <v>102</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>103</v>
-      </c>
-      <c r="B17">
-        <v>74.7</v>
       </c>
     </row>
   </sheetData>
@@ -5648,20 +5637,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B063A3DA-1C44-4C3A-8C1B-E2761804D2D3}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5675,7 +5664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5689,7 +5678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5703,7 +5692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5717,7 +5706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -5731,7 +5720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -5745,7 +5734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -5759,7 +5748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -5773,7 +5762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -5787,7 +5776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -5801,7 +5790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -5815,7 +5804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -5829,7 +5818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -5843,27 +5832,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -5878,7 +5867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -5893,7 +5882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -5901,7 +5890,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -5917,20 +5906,20 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E85C9EF-C938-4332-9062-B90E5391A4C9}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -5944,7 +5933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -5958,7 +5947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -5972,7 +5961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5986,7 +5975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -6000,7 +5989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6014,7 +6003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6028,7 +6017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6042,7 +6031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -6056,7 +6045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -6070,7 +6059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -6084,7 +6073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6098,7 +6087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -6112,27 +6101,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -6147,7 +6136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -6162,7 +6151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -6170,7 +6159,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -6186,20 +6175,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360362D6-FEDB-4209-B94A-90E1261C03E2}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6213,7 +6202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -6227,7 +6216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -6241,7 +6230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -6255,7 +6244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -6269,7 +6258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6283,7 +6272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6297,7 +6286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6311,7 +6300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -6325,7 +6314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -6339,7 +6328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -6353,7 +6342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6367,7 +6356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -6381,27 +6370,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -6416,7 +6405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -6431,7 +6420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -6439,7 +6428,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -6455,20 +6444,20 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B113761-7CD5-4A92-9B63-87C14A162C82}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6482,7 +6471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -6496,7 +6485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -6510,7 +6499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -6524,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -6538,7 +6527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6552,7 +6541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -6566,7 +6555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6580,7 +6569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -6594,7 +6583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -6608,7 +6597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -6622,7 +6611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6636,7 +6625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -6650,27 +6639,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -6685,7 +6674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -6700,7 +6689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -6708,7 +6697,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -6724,15 +6713,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01B4DCC9-BAEB-4BE3-8071-9749F432ADAE}">
   <dimension ref="A1:D22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6746,7 +6735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -6760,7 +6749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -6774,7 +6763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -6788,7 +6777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -6802,7 +6791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -6816,7 +6805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -6830,7 +6819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -6844,7 +6833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -6858,7 +6847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -6872,7 +6861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -6886,7 +6875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -6900,7 +6889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -6914,27 +6903,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -6949,7 +6938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -6964,7 +6953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -6972,7 +6961,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>77</v>
       </c>
@@ -6988,20 +6977,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42B7BCB8-2BE9-44FE-9BA0-E5BC0BEA7660}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -7015,7 +7004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -7029,7 +7018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -7043,7 +7032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -7057,7 +7046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7071,7 +7060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -7085,7 +7074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -7099,7 +7088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -7113,7 +7102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -7127,7 +7116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -7141,7 +7130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -7155,7 +7144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -7169,7 +7158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -7183,27 +7172,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -7218,7 +7207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -7233,7 +7222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -7241,7 +7230,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -7257,20 +7246,20 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C644951-C62A-48BD-BE1E-F3508FF13797}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="1.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.61328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="1.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -7284,7 +7273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -7298,7 +7287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -7312,7 +7301,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -7326,7 +7315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -7340,7 +7329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -7354,7 +7343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -7368,7 +7357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -7382,7 +7371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -7396,7 +7385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -7410,7 +7399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -7424,7 +7413,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -7438,7 +7427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -7452,27 +7441,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -7487,7 +7476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -7502,7 +7491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>71</v>
       </c>
@@ -7510,7 +7499,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>77</v>
       </c>

</xml_diff>